<commit_message>
Modif interface + debug load all equipment
</commit_message>
<xml_diff>
--- a/data/Data_cards.xlsx
+++ b/data/Data_cards.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Python\periples\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B39CE917-E2BA-43D5-9C7E-30B01E5118AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DA14694-CD19-456E-9928-6983D7F2713B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="285">
   <si>
     <t>Nom</t>
   </si>
@@ -872,23 +872,23 @@
     <t>O-75</t>
   </si>
   <si>
-    <t>type</t>
-  </si>
-  <si>
-    <t>Armes</t>
-  </si>
-  <si>
-    <t>Armures</t>
-  </si>
-  <si>
-    <t>Accessoire</t>
+    <t>arme</t>
+  </si>
+  <si>
+    <t>armure</t>
+  </si>
+  <si>
+    <t>accessoire</t>
+  </si>
+  <si>
+    <t>Type</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -905,6 +905,12 @@
     <font>
       <b/>
       <sz val="14"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -983,7 +989,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1007,7 +1013,10 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1602,10 +1611,10 @@
         <v>3</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
         <v>188</v>
       </c>
@@ -1631,10 +1640,10 @@
         <v>0</v>
       </c>
       <c r="I2" s="8" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
         <v>189</v>
       </c>
@@ -1659,11 +1668,11 @@
       <c r="H3" s="1">
         <v>0</v>
       </c>
-      <c r="I3" s="1" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I3" s="8" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
         <v>190</v>
       </c>
@@ -1688,11 +1697,11 @@
       <c r="H4" s="1">
         <v>0</v>
       </c>
-      <c r="I4" s="1" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I4" s="8" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
         <v>191</v>
       </c>
@@ -1717,11 +1726,11 @@
       <c r="H5" s="1">
         <v>0</v>
       </c>
-      <c r="I5" s="1" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I5" s="8" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
         <v>192</v>
       </c>
@@ -1746,11 +1755,11 @@
       <c r="H6" s="1">
         <v>0</v>
       </c>
-      <c r="I6" s="1" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I6" s="8" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
         <v>193</v>
       </c>
@@ -1775,11 +1784,11 @@
       <c r="H7" s="1">
         <v>0</v>
       </c>
-      <c r="I7" s="1" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I7" s="8" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
         <v>194</v>
       </c>
@@ -1804,11 +1813,11 @@
       <c r="H8" s="1">
         <v>0</v>
       </c>
-      <c r="I8" s="1" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I8" s="8" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
         <v>195</v>
       </c>
@@ -1833,11 +1842,11 @@
       <c r="H9" s="1">
         <v>0</v>
       </c>
-      <c r="I9" s="1" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I9" s="8" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
         <v>196</v>
       </c>
@@ -1862,8 +1871,11 @@
       <c r="H10" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I10" s="9" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
         <v>197</v>
       </c>
@@ -1888,11 +1900,11 @@
       <c r="H11" s="1">
         <v>0</v>
       </c>
-      <c r="I11" s="1" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I11" s="9" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
         <v>198</v>
       </c>
@@ -1917,11 +1929,11 @@
       <c r="H12" s="1">
         <v>0</v>
       </c>
-      <c r="I12" s="1" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I12" s="9" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
         <v>199</v>
       </c>
@@ -1946,11 +1958,11 @@
       <c r="H13" s="1">
         <v>0</v>
       </c>
-      <c r="I13" s="1" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I13" s="9" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
         <v>200</v>
       </c>
@@ -1975,11 +1987,11 @@
       <c r="H14" s="1">
         <v>0</v>
       </c>
-      <c r="I14" s="1" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I14" s="9" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">
         <v>201</v>
       </c>
@@ -2004,8 +2016,11 @@
       <c r="H15" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I15" s="8" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16" s="5" t="s">
         <v>202</v>
       </c>
@@ -2030,8 +2045,11 @@
       <c r="H16" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I16" s="8" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" s="5" t="s">
         <v>203</v>
       </c>
@@ -2056,8 +2074,11 @@
       <c r="H17" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I17" s="8" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18" s="5" t="s">
         <v>204</v>
       </c>
@@ -2082,8 +2103,11 @@
       <c r="H18" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I18" s="8" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A19" s="5" t="s">
         <v>205</v>
       </c>
@@ -2108,8 +2132,11 @@
       <c r="H19" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I19" s="8" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20" s="5" t="s">
         <v>206</v>
       </c>
@@ -2134,8 +2161,11 @@
       <c r="H20" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I20" s="8" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A21" s="5" t="s">
         <v>207</v>
       </c>
@@ -2160,8 +2190,11 @@
       <c r="H21" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I21" s="8" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A22" s="5" t="s">
         <v>243</v>
       </c>
@@ -2186,8 +2219,11 @@
       <c r="H22" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I22" s="8" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A23" s="5" t="s">
         <v>208</v>
       </c>
@@ -2212,8 +2248,11 @@
       <c r="H23" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I23" s="8" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A24" s="5" t="s">
         <v>209</v>
       </c>
@@ -2238,8 +2277,11 @@
       <c r="H24" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I24" s="8" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A25" s="5" t="s">
         <v>224</v>
       </c>
@@ -2264,8 +2306,11 @@
       <c r="H25" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I25" s="8" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A26" s="5" t="s">
         <v>225</v>
       </c>
@@ -2290,8 +2335,11 @@
       <c r="H26" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I26" s="8" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A27" s="5" t="s">
         <v>226</v>
       </c>
@@ -2316,11 +2364,11 @@
       <c r="H27" s="1">
         <v>0</v>
       </c>
-      <c r="I27" s="1" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I27" s="9" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A28" s="5" t="s">
         <v>227</v>
       </c>
@@ -2345,11 +2393,11 @@
       <c r="H28" s="1">
         <v>0</v>
       </c>
-      <c r="I28" s="1" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I28" s="9" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A29" s="5" t="s">
         <v>228</v>
       </c>
@@ -2374,11 +2422,11 @@
       <c r="H29" s="1">
         <v>0</v>
       </c>
-      <c r="I29" s="1" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I29" s="9" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A30" s="5" t="s">
         <v>229</v>
       </c>
@@ -2403,11 +2451,11 @@
       <c r="H30" s="1">
         <v>0</v>
       </c>
-      <c r="I30" s="1" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I30" s="9" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A31" s="5" t="s">
         <v>230</v>
       </c>
@@ -2432,11 +2480,11 @@
       <c r="H31" s="1">
         <v>0</v>
       </c>
-      <c r="I31" s="1" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I31" s="9" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A32" s="5" t="s">
         <v>231</v>
       </c>
@@ -2461,11 +2509,11 @@
       <c r="H32" s="1">
         <v>0</v>
       </c>
-      <c r="I32" s="1" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I32" s="9" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A33" s="5" t="s">
         <v>232</v>
       </c>
@@ -2490,11 +2538,11 @@
       <c r="H33" s="1">
         <v>0</v>
       </c>
-      <c r="I33" s="1" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I33" s="9" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A34" s="5" t="s">
         <v>233</v>
       </c>
@@ -2519,11 +2567,11 @@
       <c r="H34" s="1">
         <v>0</v>
       </c>
-      <c r="I34" s="1" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I34" s="9" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A35" s="5" t="s">
         <v>234</v>
       </c>
@@ -2548,11 +2596,11 @@
       <c r="H35" s="1">
         <v>0</v>
       </c>
-      <c r="I35" s="1" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I35" s="9" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A36" s="5" t="s">
         <v>235</v>
       </c>
@@ -2577,11 +2625,11 @@
       <c r="H36" s="1">
         <v>0</v>
       </c>
-      <c r="I36" s="1" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I36" s="9" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A37" s="5" t="s">
         <v>236</v>
       </c>
@@ -2606,11 +2654,11 @@
       <c r="H37" s="1">
         <v>2</v>
       </c>
-      <c r="I37" s="1" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I37" s="9" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A38" s="5" t="s">
         <v>237</v>
       </c>
@@ -2635,11 +2683,11 @@
       <c r="H38" s="1">
         <v>0</v>
       </c>
-      <c r="I38" s="1" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I38" s="9" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A39" s="5" t="s">
         <v>238</v>
       </c>
@@ -2664,11 +2712,11 @@
       <c r="H39" s="1">
         <v>0</v>
       </c>
-      <c r="I39" s="1" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I39" s="9" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A40" s="5" t="s">
         <v>239</v>
       </c>
@@ -2693,11 +2741,11 @@
       <c r="H40" s="1">
         <v>0</v>
       </c>
-      <c r="I40" s="1" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I40" s="9" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A41" s="5" t="s">
         <v>255</v>
       </c>
@@ -2722,11 +2770,11 @@
       <c r="H41" s="1">
         <v>0</v>
       </c>
-      <c r="I41" s="1" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I41" s="9" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A42" s="5" t="s">
         <v>260</v>
       </c>
@@ -2751,11 +2799,11 @@
       <c r="H42" s="1">
         <v>2</v>
       </c>
-      <c r="I42" s="1" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I42" s="9" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A43" s="5" t="s">
         <v>261</v>
       </c>
@@ -2780,11 +2828,11 @@
       <c r="H43" s="1">
         <v>0</v>
       </c>
-      <c r="I43" s="1" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I43" s="9" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A44" s="5" t="s">
         <v>262</v>
       </c>
@@ -2809,11 +2857,11 @@
       <c r="H44" s="1">
         <v>0</v>
       </c>
-      <c r="I44" s="1" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I44" s="9" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A45" s="5" t="s">
         <v>263</v>
       </c>
@@ -2838,11 +2886,11 @@
       <c r="H45" s="1">
         <v>0</v>
       </c>
-      <c r="I45" s="1" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I45" s="9" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A46" s="5" t="s">
         <v>279</v>
       </c>
@@ -2867,11 +2915,11 @@
       <c r="H46" s="1">
         <v>0</v>
       </c>
-      <c r="I46" s="1" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I46" s="8" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A47" s="5" t="s">
         <v>280</v>
       </c>
@@ -2896,11 +2944,11 @@
       <c r="H47" s="1">
         <v>0</v>
       </c>
-      <c r="I47" s="1" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I47" s="9" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A48" s="5" t="s">
         <v>269</v>
       </c>
@@ -2925,11 +2973,11 @@
       <c r="H48" s="1">
         <v>0</v>
       </c>
-      <c r="I48" s="1" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I48" s="8" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A49" s="5" t="s">
         <v>270</v>
       </c>
@@ -2954,11 +3002,11 @@
       <c r="H49" s="1">
         <v>0</v>
       </c>
-      <c r="I49" s="1" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I49" s="8" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A50" s="5" t="s">
         <v>274</v>
       </c>
@@ -2983,11 +3031,11 @@
       <c r="H50" s="1">
         <v>0</v>
       </c>
-      <c r="I50" s="1" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I50" s="9" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A51" s="5" t="s">
         <v>275</v>
       </c>
@@ -3012,11 +3060,11 @@
       <c r="H51" s="1">
         <v>0</v>
       </c>
-      <c r="I51" s="1" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I51" s="8" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A52" s="5" t="s">
         <v>276</v>
       </c>
@@ -3041,11 +3089,11 @@
       <c r="H52" s="1">
         <v>0</v>
       </c>
-      <c r="I52" s="1" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I52" s="9" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A53" s="5" t="s">
         <v>277</v>
       </c>
@@ -3070,8 +3118,8 @@
       <c r="H53" s="1">
         <v>2</v>
       </c>
-      <c r="I53" s="1" t="s">
-        <v>284</v>
+      <c r="I53" s="9" t="s">
+        <v>283</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.25">

</xml_diff>